<commit_message>
Updated life history traits for Chalcidoidea
</commit_message>
<xml_diff>
--- a/source_data/Chalcidoidea_life_history_traits.xlsx
+++ b/source_data/Chalcidoidea_life_history_traits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronquist/dev/ms-repos-iba/paper-mg-insects/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B3F422B-CCAA-1745-863C-3C14957E0085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D2BAEEB-1117-F842-A26D-585AE7B6D1D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4240" yWindow="6360" windowWidth="24820" windowHeight="17180" xr2:uid="{8F68FF23-D21D-CE4C-817A-FF9FC30FD1C7}"/>
+    <workbookView xWindow="3980" yWindow="820" windowWidth="24820" windowHeight="17180" xr2:uid="{8F68FF23-D21D-CE4C-817A-FF9FC30FD1C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -118,15 +118,9 @@
     <t>Eunotidae</t>
   </si>
   <si>
-    <t>eupelmid clade</t>
-  </si>
-  <si>
     <t>Eurytomidae</t>
   </si>
   <si>
-    <t>gall clade</t>
-  </si>
-  <si>
     <t>Herbertiidae</t>
   </si>
   <si>
@@ -166,15 +160,9 @@
     <t>Pirenidae</t>
   </si>
   <si>
-    <t>planidial clade</t>
-  </si>
-  <si>
     <t>Pteromalidae</t>
   </si>
   <si>
-    <t>Rivasia i.s.</t>
-  </si>
-  <si>
     <t>Storyeinae</t>
   </si>
   <si>
@@ -203,12 +191,6 @@
   </si>
   <si>
     <t>Ooderini associated with hosts in wood</t>
-  </si>
-  <si>
-    <t>megastigmid clade</t>
-  </si>
-  <si>
-    <t>neanastatid clade</t>
   </si>
   <si>
     <t>?</t>
@@ -354,6 +336,24 @@
   </si>
   <si>
     <t>Phytophage/Phytophage-parasitoid?</t>
+  </si>
+  <si>
+    <t>eupelmid_clade</t>
+  </si>
+  <si>
+    <t>gall_clade</t>
+  </si>
+  <si>
+    <t>megastigmid_clade</t>
+  </si>
+  <si>
+    <t>neanastatid_clade</t>
+  </si>
+  <si>
+    <t>planidial_clade</t>
+  </si>
+  <si>
+    <t>Rivasia</t>
   </si>
 </sst>
 </file>
@@ -818,13 +818,13 @@
         <v>11</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -835,10 +835,10 @@
         <v>7</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -871,7 +871,7 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
@@ -882,7 +882,7 @@
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -893,7 +893,7 @@
         <v>7</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="34" x14ac:dyDescent="0.2">
@@ -907,7 +907,7 @@
         <v>5</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -918,7 +918,7 @@
         <v>7</v>
       </c>
       <c r="C14" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="34" x14ac:dyDescent="0.2">
@@ -926,13 +926,13 @@
         <v>20</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C15" t="s">
         <v>5</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
@@ -973,13 +973,13 @@
         <v>24</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C19" t="s">
         <v>5</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -1006,7 +1006,7 @@
     </row>
     <row r="22" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
       <c r="B22" t="s">
         <v>7</v>
@@ -1015,12 +1015,12 @@
         <v>5</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B23" t="s">
         <v>7</v>
@@ -1031,21 +1031,21 @@
     </row>
     <row r="24" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>29</v>
+        <v>67</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C24" t="s">
         <v>5</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B25" t="s">
         <v>7</v>
@@ -1056,7 +1056,7 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B26" t="s">
         <v>7</v>
@@ -1067,7 +1067,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B27" t="s">
         <v>7</v>
@@ -1078,7 +1078,7 @@
     </row>
     <row r="28" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B28" t="s">
         <v>7</v>
@@ -1087,34 +1087,34 @@
         <v>5</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B29" t="s">
         <v>7</v>
       </c>
       <c r="C29" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B30" t="s">
         <v>7</v>
       </c>
       <c r="C30" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="B31" t="s">
         <v>7</v>
@@ -1123,26 +1123,26 @@
         <v>5</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C32" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B33" t="s">
         <v>7</v>
@@ -1153,7 +1153,7 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B34" t="s">
         <v>7</v>
@@ -1164,7 +1164,7 @@
     </row>
     <row r="35" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="B35" t="s">
         <v>7</v>
@@ -1173,12 +1173,12 @@
         <v>5</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B36" t="s">
         <v>7</v>
@@ -1189,7 +1189,7 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B37" t="s">
         <v>7</v>
@@ -1200,21 +1200,21 @@
     </row>
     <row r="38" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B38" t="s">
         <v>7</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B39" t="s">
         <v>7</v>
@@ -1223,26 +1223,26 @@
         <v>5</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="85" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B41" t="s">
         <v>7</v>
@@ -1251,12 +1251,12 @@
         <v>5</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="B42" t="s">
         <v>4</v>
@@ -1267,35 +1267,35 @@
     </row>
     <row r="43" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C43" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="C44" t="s">
         <v>5</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B45" t="s">
         <v>7</v>
@@ -1306,7 +1306,7 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B46" t="s">
         <v>7</v>
@@ -1317,7 +1317,7 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B47" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
Minor corrections to Chalcidoidea source data
</commit_message>
<xml_diff>
--- a/source_data/Chalcidoidea_life_history_traits.xlsx
+++ b/source_data/Chalcidoidea_life_history_traits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronquist/dev/ms-repos-iba/paper-mg-insects/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D2BAEEB-1117-F842-A26D-585AE7B6D1D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6F74547-62E6-184A-86F1-065D09B0080B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3980" yWindow="820" windowWidth="24820" windowHeight="17180" xr2:uid="{8F68FF23-D21D-CE4C-817A-FF9FC30FD1C7}"/>
+    <workbookView xWindow="3020" yWindow="500" windowWidth="24820" windowHeight="17180" xr2:uid="{8F68FF23-D21D-CE4C-817A-FF9FC30FD1C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="88">
   <si>
     <t>Clade</t>
   </si>
@@ -354,6 +354,54 @@
   </si>
   <si>
     <t>Rivasia</t>
+  </si>
+  <si>
+    <t>Family</t>
+  </si>
+  <si>
+    <t>Azotidae;Signiphoridae</t>
+  </si>
+  <si>
+    <t>Chalcididae</t>
+  </si>
+  <si>
+    <t>Asaphesinae_i_s</t>
+  </si>
+  <si>
+    <t>Ormyridae;Cynipencyrtidae;Tanaostigmatidae;Melanosomellidae;Epichrysomallidae</t>
+  </si>
+  <si>
+    <t>Leucospidae;Ooderidae</t>
+  </si>
+  <si>
+    <t>Metapelmatidae;Megastigmidae</t>
+  </si>
+  <si>
+    <t>Neanastatidae_s_lat</t>
+  </si>
+  <si>
+    <t>Rivasia_i_s</t>
+  </si>
+  <si>
+    <t>Storyeinae_i_s</t>
+  </si>
+  <si>
+    <t>Micradellinae_i_s</t>
+  </si>
+  <si>
+    <t>Ennogerinae_i_s</t>
+  </si>
+  <si>
+    <t>Eopelma_i_s</t>
+  </si>
+  <si>
+    <t>Neapterolelapinae_i_s</t>
+  </si>
+  <si>
+    <t>Eucharitidae;Chrysolampidae;Perilampidae;Eutrichosomatidae;Spalangiidae</t>
+  </si>
+  <si>
+    <t>Eupelmidae;Heydeniidae;Lyciscidae;Ditropinotellinae</t>
   </si>
 </sst>
 </file>
@@ -418,7 +466,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -430,6 +478,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -746,583 +797,725 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52709545-EF23-7842-8BB1-34DBB6C71382}">
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="33" customWidth="1"/>
-    <col min="3" max="3" width="20.1640625" customWidth="1"/>
-    <col min="4" max="4" width="77.5" style="6" customWidth="1"/>
+    <col min="1" max="1" width="29.33203125" style="6" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="33" customWidth="1"/>
+    <col min="4" max="4" width="20.1640625" customWidth="1"/>
+    <col min="5" max="5" width="77.5" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
-        <v>7</v>
+      <c r="B3" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
       <c r="C4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
       <c r="C5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A7" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="3" t="s">
+      <c r="B7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A8" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B8" t="s">
-        <v>7</v>
+      <c r="B8" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A9" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B9" t="s">
-        <v>7</v>
+      <c r="B9" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A10" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B10" t="s">
-        <v>7</v>
+      <c r="B10" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="C10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A11" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B11" t="s">
-        <v>7</v>
+      <c r="B11" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="C11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
+    <row r="12" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A12" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B12" t="s">
-        <v>7</v>
-      </c>
       <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A13" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B13" t="s">
-        <v>7</v>
-      </c>
       <c r="C13" t="s">
-        <v>5</v>
-      </c>
-      <c r="D13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" t="s">
+        <v>5</v>
+      </c>
+      <c r="E13" s="4" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
+    <row r="14" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A14" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B14" t="s">
-        <v>7</v>
+      <c r="B14" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="C14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
+    <row r="15" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A15" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C15" t="s">
-        <v>5</v>
-      </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E15" s="4" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
+    <row r="16" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A16" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B16" t="s">
-        <v>7</v>
+      <c r="B16" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="C16" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D16" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A17" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B17" t="s">
-        <v>7</v>
+      <c r="B17" s="2" t="s">
+        <v>22</v>
       </c>
       <c r="C17" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A18" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B18" t="s">
-        <v>7</v>
-      </c>
       <c r="C18" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A19" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C19" t="s">
-        <v>5</v>
-      </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" t="s">
+        <v>5</v>
+      </c>
+      <c r="E19" s="4" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
+    <row r="20" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A20" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B20" t="s">
-        <v>7</v>
+      <c r="B20" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="C20" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A21" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B21" t="s">
-        <v>7</v>
+      <c r="B21" s="2" t="s">
+        <v>26</v>
       </c>
       <c r="C21" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A22" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A22" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B22" t="s">
-        <v>7</v>
-      </c>
       <c r="C22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" t="s">
+        <v>5</v>
+      </c>
+      <c r="E22" s="4" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="2" t="s">
+    <row r="23" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A23" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B23" t="s">
-        <v>7</v>
+      <c r="B23" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="C23" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A24" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="C24" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C24" t="s">
-        <v>5</v>
-      </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" t="s">
+        <v>5</v>
+      </c>
+      <c r="E24" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="2" t="s">
+    <row r="25" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A25" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B25" t="s">
-        <v>7</v>
+      <c r="B25" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="C25" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A26" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B26" t="s">
-        <v>7</v>
+      <c r="B26" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="C26" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A27" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B27" t="s">
-        <v>7</v>
+      <c r="B27" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="C27" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A28" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A28" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B28" t="s">
-        <v>7</v>
-      </c>
       <c r="C28" t="s">
-        <v>5</v>
-      </c>
-      <c r="D28" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" t="s">
+        <v>5</v>
+      </c>
+      <c r="E28" s="4" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="2" t="s">
+    <row r="29" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A29" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B29" t="s">
-        <v>7</v>
+      <c r="B29" s="2" t="s">
+        <v>32</v>
       </c>
       <c r="C29" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="2" t="s">
+    <row r="30" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A30" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B30" t="s">
-        <v>7</v>
+      <c r="B30" s="2" t="s">
+        <v>33</v>
       </c>
       <c r="C30" t="s">
+        <v>7</v>
+      </c>
+      <c r="D30" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A31" s="2" t="s">
+    <row r="31" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A31" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B31" t="s">
-        <v>7</v>
-      </c>
       <c r="C31" t="s">
-        <v>5</v>
-      </c>
-      <c r="D31" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D31" t="s">
+        <v>5</v>
+      </c>
+      <c r="E31" s="4" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A32" s="2" t="s">
+    <row r="32" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A32" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="C32" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>52</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="E32" s="4" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="2" t="s">
+    <row r="33" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A33" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B33" t="s">
-        <v>7</v>
+      <c r="B33" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="C33" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D33" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A34" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B34" t="s">
-        <v>7</v>
+      <c r="B34" s="2" t="s">
+        <v>36</v>
       </c>
       <c r="C34" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A35" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A35" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B35" t="s">
-        <v>7</v>
-      </c>
       <c r="C35" t="s">
-        <v>5</v>
-      </c>
-      <c r="D35" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" t="s">
+        <v>5</v>
+      </c>
+      <c r="E35" s="4" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="2" t="s">
+    <row r="36" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A36" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B36" t="s">
-        <v>7</v>
-      </c>
       <c r="C36" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A37" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B37" t="s">
-        <v>7</v>
+      <c r="B37" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="C37" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A38" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A38" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B38" t="s">
-        <v>7</v>
-      </c>
-      <c r="C38" s="3" t="s">
+      <c r="B38" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C38" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D38" s="4" t="s">
+      <c r="E38" s="4" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A39" s="2" t="s">
+    <row r="39" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A39" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B39" t="s">
-        <v>7</v>
+      <c r="B39" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="C39" t="s">
-        <v>5</v>
-      </c>
-      <c r="D39" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39" t="s">
+        <v>5</v>
+      </c>
+      <c r="E39" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="85" x14ac:dyDescent="0.2">
-      <c r="A40" s="2" t="s">
+    <row r="40" spans="1:5" ht="85" x14ac:dyDescent="0.2">
+      <c r="A40" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="C40" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="D40" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="D40" s="4" t="s">
+      <c r="E40" s="4" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A41" s="2" t="s">
+    <row r="41" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A41" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B41" t="s">
-        <v>7</v>
+      <c r="B41" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="C41" t="s">
-        <v>5</v>
-      </c>
-      <c r="D41" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" t="s">
+        <v>5</v>
+      </c>
+      <c r="E41" s="4" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="2" t="s">
+    <row r="42" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A42" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" t="s">
         <v>4</v>
       </c>
-      <c r="C42" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A43" s="2" t="s">
+      <c r="D42" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A43" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="B43" t="s">
-        <v>52</v>
       </c>
       <c r="C43" t="s">
         <v>52</v>
       </c>
-      <c r="D43" s="6" t="s">
+      <c r="D43" t="s">
+        <v>52</v>
+      </c>
+      <c r="E43" s="6" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A44" s="2" t="s">
+    <row r="44" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A44" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B44" s="3" t="s">
+      <c r="B44" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C44" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C44" t="s">
-        <v>5</v>
-      </c>
-      <c r="D44" s="4" t="s">
+      <c r="D44" t="s">
+        <v>5</v>
+      </c>
+      <c r="E44" s="4" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="2" t="s">
+    <row r="45" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A45" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B45" t="s">
-        <v>7</v>
+      <c r="B45" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="C45" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D45" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A46" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B46" t="s">
-        <v>7</v>
+      <c r="B46" s="2" t="s">
+        <v>45</v>
       </c>
       <c r="C46" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D46" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A47" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B47" t="s">
-        <v>7</v>
+      <c r="B47" s="2" t="s">
+        <v>46</v>
       </c>
       <c r="C47" t="s">
+        <v>7</v>
+      </c>
+      <c r="D47" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Minor update to chalcidoid taxonomy and trait data
</commit_message>
<xml_diff>
--- a/source_data/Chalcidoidea_life_history_traits.xlsx
+++ b/source_data/Chalcidoidea_life_history_traits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronquist/dev/ms-repos-iba/paper-mg-insects/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6F74547-62E6-184A-86F1-065D09B0080B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC92504B-448D-A84B-8B18-61F4A3FA5083}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3020" yWindow="500" windowWidth="24820" windowHeight="17180" xr2:uid="{8F68FF23-D21D-CE4C-817A-FF9FC30FD1C7}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="89">
   <si>
     <t>Clade</t>
   </si>
@@ -374,9 +374,6 @@
     <t>Leucospidae;Ooderidae</t>
   </si>
   <si>
-    <t>Metapelmatidae;Megastigmidae</t>
-  </si>
-  <si>
     <t>Neanastatidae_s_lat</t>
   </si>
   <si>
@@ -402,6 +399,12 @@
   </si>
   <si>
     <t>Eupelmidae;Heydeniidae;Lyciscidae;Ditropinotellinae</t>
+  </si>
+  <si>
+    <t>Metapelmatidae</t>
+  </si>
+  <si>
+    <t>Megastigmidae_s_lat</t>
   </si>
 </sst>
 </file>
@@ -797,7 +800,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52709545-EF23-7842-8BB1-34DBB6C71382}">
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.33203125" style="6" customWidth="1"/>
@@ -1062,7 +1065,7 @@
     </row>
     <row r="18" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>23</v>
@@ -1076,7 +1079,7 @@
     </row>
     <row r="19" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>24</v>
@@ -1121,7 +1124,7 @@
     </row>
     <row r="22" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>66</v>
@@ -1256,7 +1259,7 @@
     </row>
     <row r="31" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>68</v>
@@ -1273,41 +1276,41 @@
     </row>
     <row r="32" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" s="7" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>47</v>
+        <v>87</v>
+      </c>
+      <c r="C32" t="s">
+        <v>7</v>
       </c>
       <c r="D32" t="s">
-        <v>52</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="s">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C33" t="s">
-        <v>7</v>
+        <v>34</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>47</v>
       </c>
       <c r="D33" t="s">
-        <v>5</v>
+        <v>52</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A34" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C34" t="s">
         <v>7</v>
@@ -1318,41 +1321,41 @@
     </row>
     <row r="35" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" s="7" t="s">
-        <v>79</v>
+        <v>36</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>69</v>
+        <v>36</v>
       </c>
       <c r="C35" t="s">
         <v>7</v>
       </c>
       <c r="D35" t="s">
         <v>5</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>37</v>
+        <v>69</v>
       </c>
       <c r="C36" t="s">
         <v>7</v>
       </c>
       <c r="D36" t="s">
         <v>5</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C37" t="s">
         <v>7</v>
@@ -1363,140 +1366,140 @@
     </row>
     <row r="38" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C38" t="s">
         <v>7</v>
       </c>
-      <c r="D38" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>48</v>
+      <c r="D38" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C39" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A40" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B40" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C39" t="s">
-        <v>7</v>
-      </c>
-      <c r="D39" t="s">
-        <v>5</v>
-      </c>
-      <c r="E39" s="4" t="s">
+      <c r="C40" t="s">
+        <v>7</v>
+      </c>
+      <c r="D40" t="s">
+        <v>5</v>
+      </c>
+      <c r="E40" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="85" x14ac:dyDescent="0.2">
-      <c r="A40" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="B40" s="2" t="s">
+    <row r="41" spans="1:5" ht="85" x14ac:dyDescent="0.2">
+      <c r="A41" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="C41" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="D41" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E40" s="4" t="s">
+      <c r="E41" s="4" t="s">
         <v>53</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A41" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C41" t="s">
-        <v>7</v>
-      </c>
-      <c r="D41" t="s">
-        <v>5</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="s">
-        <v>80</v>
+        <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>71</v>
+        <v>41</v>
       </c>
       <c r="C42" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D42" t="s">
         <v>5</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" s="7" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>42</v>
+        <v>71</v>
       </c>
       <c r="C43" t="s">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="D43" t="s">
-        <v>52</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" s="7" t="s">
-        <v>43</v>
+        <v>80</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>65</v>
+        <v>42</v>
+      </c>
+      <c r="C44" t="s">
+        <v>52</v>
       </c>
       <c r="D44" t="s">
-        <v>5</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C45" t="s">
-        <v>7</v>
+        <v>43</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>65</v>
       </c>
       <c r="D45" t="s">
         <v>5</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A46" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C46" t="s">
         <v>7</v>
@@ -1507,15 +1510,29 @@
     </row>
     <row r="47" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C47" t="s">
+        <v>7</v>
+      </c>
+      <c r="D47" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A48" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B48" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C47" t="s">
-        <v>7</v>
-      </c>
-      <c r="D47" t="s">
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>